<commit_message>
feat: agregar scraper de expedientes PJN con extracción de últimos movimientos
</commit_message>
<xml_diff>
--- a/expedientes_pjn.xlsx
+++ b/expedientes_pjn.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,27 +417,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Número de expediente</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Juzgado</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Carátula</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Situación</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Últ. Act. listado</t>
         </is>
@@ -458,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CSS 025528/1990</t>
+          <t>CSS 014356/2012</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CAMARA FEDERAL DE LA SEGURIDAD SOCIAL - SALA 3</t>
+          <t>JUZGADO FEDERAL DE SANTA FE 2</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AIMAR DE VODOPIA CELINA C/ INPS-COMISION NACIONAL DE PREVISION SOCIAL S/REAJUSTES VARIOS</t>
+          <t>ARIETTO RAUL AMERICO C/ ANSES S/REAJUSTES VARIOS</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -478,78 +466,78 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>6/05/1992</t>
+          <t>29/05/2014</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FRO 003835/2016</t>
+          <t>CSS 029579/1990</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>JUZGADO FEDERAL DE SANTA FE 1 - SECRETARIA LEYES ESPECIALES</t>
+          <t>CAMARA FEDERAL DE LA SEGURIDAD SOCIAL - SALA 1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AIMARETTI, VALENTIN JOSE C/ ANSES S/REAJUSTES POR MOVILIDAD</t>
+          <t>ABRAHAN JULIO C/ INPS-COMISION NACIONAL DE PREVISION SOCIAL S/REAJUSTES VARIOS</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>EN LETRA</t>
+          <t>EN DESPACHO</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>14/05/2018</t>
+          <t>7/06/2015</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>52000611/2010</t>
+          <t>CSS 004074/2001</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>JUZGADO FEDERAL DE SANTA FE 1 - SECRETARIA CIVIL Y COMERCIAL</t>
+          <t>JUZGADO FEDERAL DE SANTA FE 2</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AKEL, IRMA JOSEFA C/ ANSES S/REAJUSTES POR MOVILIDAD</t>
+          <t>ABSI SYLVIA BEATRIZ C/ ANSES S/REAJUSTES VARIOS</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>EN LETRA</t>
+          <t>EN DESPACHO</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>23/08/2017</t>
+          <t>5/02/2003</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CSS 072781/2012</t>
+          <t>62000991/2011</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CAMARA FEDERAL DE ROSARIO - MESA DE ENTRADAS SANTA FE - 1RA INSTANCIA</t>
+          <t>JUZGADO FEDERAL DE SANTA FE 2 - SECRETARIA CIVIL Y COMERCIAL</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AKEL IRMA JOSEFA C/ ANSES S/REAJUSTES VARIOS</t>
+          <t>ACASTELLO, ETHEL MAGDALENA C/ A.N.SE.S. S/REAJUSTES VARIOS</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -559,68 +547,68 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>22/05/2014</t>
+          <t>4/08/2025</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CSS 047538/2008</t>
+          <t>FRO 001297/2013</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAMARA FEDERAL DE ROSARIO - MESA DE ENTRADAS SANTA FE - 1RA INSTANCIA</t>
+          <t>JUZGADO FEDERAL DE SANTA FE 1 - SECRETARIA EJECUCION FISCAL</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ALANIZ DELIA DELMIRA C/ ANSES S/REAJUSTES VARIOS</t>
+          <t>ACEVEDO, ANTONIA EDITH C/ ANSES S/REAJUSTES POR MOVILIDAD</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>EN DESPACHO</t>
+          <t>EN LETRA</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>7/06/2015</t>
+          <t>14/05/2018</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FRO 017134/2016</t>
+          <t>CSS 003855/2013</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>JUZGADO FEDERAL DE RAFAELA - SECRETARIA CIVIL</t>
+          <t>JUZGADO FEDERAL DE SANTA FE 2</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ALASSIA, MIRTA ROSA DEL CARMEN C/ ANSES S/REAJUSTES VARIOS</t>
+          <t>ACEVEDO ANTONIA EDITH C/ ANSES S/REAJUSTES VARIOS</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>EN LETRA</t>
+          <t>EN DESPACHO</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>24/06/2019</t>
+          <t>2/06/2014</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CSS 013723/2012</t>
+          <t>CSS 013781/2000</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -630,7 +618,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ALBERTO HECTOR JUAN C/ ANSES S/REAJUSTES VARIOS</t>
+          <t>ACOSTA RAMON HORLANDO C/ ANSES S/REAJUSTES VARIOS</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -640,24 +628,24 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>7/06/2015</t>
+          <t>9/11/2001</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>FRO 063966/2017</t>
+          <t>52000615/2010</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>JUZGADO FEDERAL DE RAFAELA - SECRETARIA CIVIL</t>
+          <t>JUZGADO FEDERAL DE SANTA FE 1 - SECRETARIA CIVIL Y COMERCIAL</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ALBERTO, PILAR MARIA C/ ANSES S/PENSIONES</t>
+          <t>AGOSTINI, EDERMINDO JOSE C/ ANSES S/REAJUSTES POR MOVILIDAD</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -667,24 +655,24 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4/04/2023</t>
+          <t>29/08/2017</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CSS 036296/1999</t>
+          <t>CSS 066426/2012</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>JUZGADO FEDERAL DE SANTA FE 2</t>
+          <t>CAMARA FEDERAL DE ROSARIO - MESA DE ENTRADAS SANTA FE - 1RA INSTANCIA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ALBORNOZ CARLOS C/ ANSES S/REAJUSTES VARIOS</t>
+          <t>AGOSTINI EDERMINDO JOSE C/ ANSES S/REAJUSTES VARIOS</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -694,122 +682,122 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>7/06/2015</t>
+          <t>26/05/2014</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>53000369/2007</t>
+          <t>CSS 061496/1993</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>JUZGADO FEDERAL DE SANTA FE 1 - SECRETARIA LEYES ESPECIALES</t>
+          <t>CAMARA FEDERAL DE LA SEGURIDAD SOCIAL - SALA 3</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ALBORNOZ CARLOS ROLANDO C/ A.N.S.E.S. S/EJECUCIÓN PREVISIONAL</t>
+          <t>AGOSTO ELDO ANGEL C/ INPS-CAJA NAC DE PREV PARA EL PERS DEL EST Y SERV PUBL. S/REAJUSTES VARIOS</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>EN LETRA</t>
+          <t>EN DESPACHO</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>26/07/2017</t>
+          <t>21/06/1994</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CSS 077979/1994</t>
+          <t>62000540/2012</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CAMARA FEDERAL DE LA SEGURIDAD SOCIAL - SALA 3</t>
+          <t>JUZGADO FEDERAL DE SANTA FE 2</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ALCANTARA ERNESTO C/ ANSES S/REAJUSTES VARIOS</t>
+          <t>AGUILAR COOLEN, LUIS PEDRO R. C/ A.N.SE.S. S/REAJUSTES VARIOS</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>EN DESPACHO</t>
+          <t>EN LETRA</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>30/05/1995</t>
+          <t>30/05/2023</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FRO 020587/2016</t>
+          <t>CSS 032369/1993</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>JUZGADO FEDERAL DE RAFAELA - SECRETARIA CIVIL</t>
+          <t>CAMARA FEDERAL DE LA SEGURIDAD SOCIAL - SALA 3</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ALEMANI, GLADIS BEATRIZ C/ ANSES S/REAJUSTES VARIOS</t>
+          <t>AGUIRRE DE MONDINO ELSA C/ INPS-CAJA NAC DE PREV PARA EL PERS DEL EST Y SERV PUBL. S/REAJUSTES VARIOS</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>EN LETRA</t>
+          <t>EN DESPACHO</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>24/06/2019</t>
+          <t>20/04/1994</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CSS 079318/1994</t>
+          <t>62000368/2012</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CAMARA FEDERAL DE LA SEGURIDAD SOCIAL - SALA 2</t>
+          <t>JUZGADO FEDERAL DE SANTA FE 2 - SECRETARIA CIVIL Y COMERCIAL</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ALESSANDRIA DE CAMARA IGEA C/ ANSES S/REAJUSTES VARIOS</t>
+          <t>AGUIRRE, ERNESTO JOSE C/ A.N.SE.S. S/EJECUCIÓN PREVISIONAL</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>EN DESPACHO</t>
+          <t>EN LETRA</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>7/06/2015</t>
+          <t>21/02/2018</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FRO 042825/2018</t>
+          <t>FRO 003802/2014</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -819,24 +807,24 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ALESSIATO, HUGO JOSE C/ ANSES S/REAJUSTES VARIOS</t>
+          <t>AGUIRRE, LUCIA IRENE C/ ANSES S/REAJUSTES POR MOVILIDAD</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>EN LETRA</t>
+          <t>CONFRONTE</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12/02/2026</t>
+          <t>2/10/2018</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>FRO 023975/2013</t>
+          <t>53000426/2012</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -846,17 +834,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ALESSO, ALBERTO SANTIAGO C/ ANSES S/REAJUSTES POR MOVILIDAD</t>
+          <t>AGUIRRE, OLGA ESTELA C/ ANSES Y PEN /S AMPARO LEY 16986 Y M</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>EN LETRA</t>
+          <t>CONFRONTE</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>20/04/2018</t>
+          <t>2/10/2017</t>
         </is>
       </c>
     </row>

</xml_diff>